<commit_message>
Add PRS complaint translations
</commit_message>
<xml_diff>
--- a/docassemble/StudentEvaluations/data/sources/prs_complaint_interview_es.xlsx
+++ b/docassemble/StudentEvaluations/data/sources/prs_complaint_interview_es.xlsx
@@ -17428,19 +17428,19 @@
         <is>
           <t>Has subido ${ x[i].pages.num_pages() } páginas hasta ahora.
 &lt;% current_doc_size = sum(ap.size_in_bytes() for ap in x[i].pages.complete_elements()) %&gt;  
-__PROTEGIDO_7__
+% if hasattr(x, 'maximum_size_per_doc'):
 Este documento debe ser más pequeño que ${ humanize.naturalsize(x.maximum_size_per_doc) }.
-__PROTEGIDO_8__
+% if not hasattr(x, 'maximum_size') or x.maximum_size_per_doc - current_doc_size &lt; x.maximum_size - x.size_in_bytes() - current_doc_size:
 Puedes subir ${ humanize.naturalsize(x.maximum_size_per_doc - current_doc_size) } más.
-__PROTEGIDO_9__
+% else:
 Puedes subir ${ humanize.naturalsize(x.maximum_size - x.size_in_bytes() - current_doc_size) } más.
 % endif
 % endif
-__PROTEGIDO_12__
+% if hasattr(x, 'maximum_size'):
 El tamaño total de todas las exhibiciones debe ser menor que ${ humanize.naturalsize(x.maximum_size) }.
 Puedes subir ${ humanize.naturalsize(x.maximum_size - x.size_in_bytes() - current_doc_size) } más.
-__PROTEGIDO_13__
-__PROTEGIDO_6__</t>
+% endif
+${ collapse_template(x[i].in_progress_template) }</t>
         </is>
       </c>
     </row>
@@ -26943,7 +26943,7 @@
       </c>
       <c r="H608" s="3" t="inlineStr">
         <is>
-          <t>Tu idioma</t>
+          <t>Su idioma</t>
         </is>
       </c>
     </row>
@@ -26983,7 +26983,7 @@
       </c>
       <c r="H609" s="3" t="inlineStr">
         <is>
-          <t>¿Qué idioma hablas mejor?</t>
+          <t>¿Qué idioma habla mejor?</t>
         </is>
       </c>
     </row>
@@ -27023,7 +27023,7 @@
       </c>
       <c r="H610" s="3" t="inlineStr">
         <is>
-          <t>¿Cómo le informaste a la escuela sobre tus necesidades lingüísticas?</t>
+          <t>¿Cómo le informó a la escuela sobre sus necesidades de idioma?</t>
         </is>
       </c>
     </row>
@@ -27063,7 +27063,7 @@
       </c>
       <c r="H611" s="3" t="inlineStr">
         <is>
-          <t>Cuéntanos más sobre cómo la escuela supo que prefieres un idioma distinto al inglés.</t>
+          <t>Cuéntenos más sobre cómo la escuela supo que prefiere un idioma distinto al inglés.</t>
         </is>
       </c>
     </row>
@@ -27190,7 +27190,7 @@
       </c>
       <c r="H614" s="3" t="inlineStr">
         <is>
-          <t>vocación</t>
+          <t>llamada</t>
         </is>
       </c>
     </row>
@@ -30112,12 +30112,12 @@
         <is>
           <t>% if not other_document_name == "":
 % for document in translated_documents:
-El ${ document.date }, ${ school.address.name } envió un ${ noun_singular( other_document_name ).lower() } que no se tradujo a ${ parent.language }. __PROTEGIDO_4__
-__PROTEGIDO_12__
-__PROTEGIDO_13__
+El ${ document.date }, ${ school.address.name } envió un ${ noun_singular( other_document_name ).lower() } que no se tradujo a ${ parent.language }. ${ fix_punctuation(document.description) if document.description else '' }
+% endfor
+% endif
 % if other_document_name == "": 
-__PROTEGIDO_15__
-El ${ document.date }, ${ school.address.name } envió un ${ noun_singular(evaluation_options[document.name]).lower() } que no se tradujo a ${ parent.language }. __PROTEGIDO_9__
+% for document in translated_documents:
+El ${ document.date }, ${ school.address.name } envió un ${ noun_singular(evaluation_options[document.name]).lower() } que no se tradujo a ${ parent.language }. ${ fix_punctuation(document.description) if document.description else '' }
 % endfor
 % endif</t>
         </is>
@@ -30224,18 +30224,18 @@
       </c>
       <c r="H687" s="3" t="inlineStr">
         <is>
-          <t>__PROTEGIDO_6__
+          <t>% for meeting in meetings:
 El ${ meeting.date }, tuve una reunión ${ meeting.type } con ${ school.address.name } sobre ${ meeting.name }.\
-__PROTEGIDO_7__
+% if meeting.requested:
  Solicité un intérprete que hable ${ parent.language } en la reunión.\
-__PROTEGIDO_8__
-__PROTEGIDO_9__
+% endif
+% if not meeting.had_interpreter:
  No hubo ningún intérprete en la reunión.\
 % elif not meeting.interpreter_was_successful:
  La interpretación fue mala y no pude participar en la reunión.\
 % endif
- __PROTEGIDO_5__
-__PROTEGIDO_12__</t>
+ ${ fix_punctuation(meeting.description) }
+% endfor</t>
         </is>
       </c>
     </row>
@@ -30559,7 +30559,7 @@
       </c>
       <c r="H694" s="3" t="inlineStr">
         <is>
-          <t>¿Cómo te afectó que el colegio no se comunicara contigo en tu propio idioma? Utilice sus propias palabras.</t>
+          <t>¿Cómo le afectó que el colegio no se comunicara con usted en su propio idioma? Utilice sus propias palabras.</t>
         </is>
       </c>
     </row>

</xml_diff>